<commit_message>
Ajout composition 2026-10-28 15:31:01 à l'historique
</commit_message>
<xml_diff>
--- a/database_historique.xlsx
+++ b/database_historique.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,34 +491,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Match_20261028_144803</t>
+          <t>Match_20261028_153101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-28 14:48:03</t>
+          <t>2026-10-28 15:31:01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Antho, Benoit, Damien, Ioan, Joker Léo</t>
+          <t>Nico P, Cedric, Dimeh, Mex, Jonh</t>
         </is>
       </c>
       <c r="D2" t="n">
+        <v>36</v>
+      </c>
+      <c r="E2" t="n">
         <v>34</v>
       </c>
-      <c r="E2" t="n">
-        <v>32</v>
-      </c>
       <c r="F2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G2" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Nico M, Frank, Mex, Cyril B, Joker Test</t>
+          <t>David, Attou, Gabriel, Joker Léo, Joker Olive</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -528,17 +528,73 @@
         <v>33</v>
       </c>
       <c r="K2" t="n">
+        <v>29</v>
+      </c>
+      <c r="L2" t="n">
+        <v>35</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>[{"Nom du Joueur":"Nico P","Attaque":6,"D\u00e9fense":8,"Gardien":5,"Collectif":9,"Surnoms":"NicoP","is_joker":false},{"Nom du Joueur":"Cedric","Attaque":8,"D\u00e9fense":8,"Gardien":5,"Collectif":8,"Surnoms":"C\u00e9dric","is_joker":false},{"Nom du Joueur":"Dimeh","Attaque":8,"D\u00e9fense":6,"Gardien":5,"Collectif":8,"Surnoms":"Dimeh","is_joker":false},{"Nom du Joueur":"Mex","Attaque":7,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Jonh","Attaque":7,"D\u00e9fense":5,"Gardien":5,"Collectif":6,"Surnoms":"","is_joker":false}]</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>[{"Nom du Joueur":"David","Attaque":7,"D\u00e9fense":5,"Gardien":5,"Collectif":6,"Surnoms":"Dav","is_joker":false},{"Nom du Joueur":"Attou","Attaque":6,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Gabriel","Attaque":7,"D\u00e9fense":7,"Gardien":5,"Collectif":7,"Surnoms":"Gaby","is_joker":false},{"Nom du Joueur":"Joker L\u00e9o","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true},{"Nom du Joueur":"Joker Olive","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Match_20261028_144803</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-28 14:48:03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Antho, Benoit, Damien, Ioan, Joker Léo</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>34</v>
+      </c>
+      <c r="E3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F3" t="n">
         <v>27</v>
       </c>
-      <c r="L2" t="n">
+      <c r="G3" t="n">
+        <v>36</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Nico M, Frank, Mex, Cyril B, Joker Test</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>34</v>
+      </c>
+      <c r="J3" t="n">
+        <v>33</v>
+      </c>
+      <c r="K3" t="n">
+        <v>27</v>
+      </c>
+      <c r="L3" t="n">
         <v>37</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>[{"Nom du Joueur":"Antho","Attaque":5,"D\u00e9fense":5,"Gardien":5,"Collectif":5,"Surnoms":"Saumon","is_joker":false},{"Nom du Joueur":"Benoit","Attaque":6,"D\u00e9fense":5,"Gardien":5,"Collectif":7,"Surnoms":"Beny","is_joker":false},{"Nom du Joueur":"Damien","Attaque":8,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Ioan","Attaque":8,"D\u00e9fense":8,"Gardien":5,"Collectif":9,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Joker L\u00e9o","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true}]</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>[{"Nom du Joueur":"Nico M","Attaque":5,"D\u00e9fense":6,"Gardien":5,"Collectif":7,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Frank","Attaque":8,"D\u00e9fense":5,"Gardien":5,"Collectif":6,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Mex","Attaque":7,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Cyril B","Attaque":7,"D\u00e9fense":8,"Gardien":5,"Collectif":9,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Joker Test","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true}]</t>
         </is>

</xml_diff>

<commit_message>
Ajout composition 2026-10-28 15:31:02 à l'historique
</commit_message>
<xml_diff>
--- a/database_historique.xlsx
+++ b/database_historique.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Match_20261028_153101</t>
+          <t>Match_20261028_153102</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-28 15:31:01</t>
+          <t>2026-10-28 15:31:02</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -547,34 +547,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Match_20261028_144803</t>
+          <t>Match_20261028_153101</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-28 14:48:03</t>
+          <t>2026-10-28 15:31:01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Antho, Benoit, Damien, Ioan, Joker Léo</t>
+          <t>Nico P, Cedric, Dimeh, Mex, Jonh</t>
         </is>
       </c>
       <c r="D3" t="n">
+        <v>36</v>
+      </c>
+      <c r="E3" t="n">
         <v>34</v>
       </c>
-      <c r="E3" t="n">
-        <v>32</v>
-      </c>
       <c r="F3" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Nico M, Frank, Mex, Cyril B, Joker Test</t>
+          <t>David, Attou, Gabriel, Joker Léo, Joker Olive</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -584,17 +584,73 @@
         <v>33</v>
       </c>
       <c r="K3" t="n">
+        <v>29</v>
+      </c>
+      <c r="L3" t="n">
+        <v>35</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>[{"Nom du Joueur":"Nico P","Attaque":6,"D\u00e9fense":8,"Gardien":5,"Collectif":9,"Surnoms":"NicoP","is_joker":false},{"Nom du Joueur":"Cedric","Attaque":8,"D\u00e9fense":8,"Gardien":5,"Collectif":8,"Surnoms":"C\u00e9dric","is_joker":false},{"Nom du Joueur":"Dimeh","Attaque":8,"D\u00e9fense":6,"Gardien":5,"Collectif":8,"Surnoms":"Dimeh","is_joker":false},{"Nom du Joueur":"Mex","Attaque":7,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Jonh","Attaque":7,"D\u00e9fense":5,"Gardien":5,"Collectif":6,"Surnoms":"","is_joker":false}]</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>[{"Nom du Joueur":"David","Attaque":7,"D\u00e9fense":5,"Gardien":5,"Collectif":6,"Surnoms":"Dav","is_joker":false},{"Nom du Joueur":"Attou","Attaque":6,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Gabriel","Attaque":7,"D\u00e9fense":7,"Gardien":5,"Collectif":7,"Surnoms":"Gaby","is_joker":false},{"Nom du Joueur":"Joker L\u00e9o","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true},{"Nom du Joueur":"Joker Olive","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Match_20261028_144803</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-28 14:48:03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Antho, Benoit, Damien, Ioan, Joker Léo</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>34</v>
+      </c>
+      <c r="E4" t="n">
+        <v>32</v>
+      </c>
+      <c r="F4" t="n">
         <v>27</v>
       </c>
-      <c r="L3" t="n">
+      <c r="G4" t="n">
+        <v>36</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Nico M, Frank, Mex, Cyril B, Joker Test</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>34</v>
+      </c>
+      <c r="J4" t="n">
+        <v>33</v>
+      </c>
+      <c r="K4" t="n">
+        <v>27</v>
+      </c>
+      <c r="L4" t="n">
         <v>37</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>[{"Nom du Joueur":"Antho","Attaque":5,"D\u00e9fense":5,"Gardien":5,"Collectif":5,"Surnoms":"Saumon","is_joker":false},{"Nom du Joueur":"Benoit","Attaque":6,"D\u00e9fense":5,"Gardien":5,"Collectif":7,"Surnoms":"Beny","is_joker":false},{"Nom du Joueur":"Damien","Attaque":8,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Ioan","Attaque":8,"D\u00e9fense":8,"Gardien":5,"Collectif":9,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Joker L\u00e9o","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true}]</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>[{"Nom du Joueur":"Nico M","Attaque":5,"D\u00e9fense":6,"Gardien":5,"Collectif":7,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Frank","Attaque":8,"D\u00e9fense":5,"Gardien":5,"Collectif":6,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Mex","Attaque":7,"D\u00e9fense":7,"Gardien":5,"Collectif":8,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Cyril B","Attaque":7,"D\u00e9fense":8,"Gardien":5,"Collectif":9,"Surnoms":"","is_joker":false},{"Nom du Joueur":"Joker Test","Attaque":7,"D\u00e9fense":7,"Gardien":7,"Collectif":7,"Surnoms":"","is_joker":true}]</t>
         </is>

</xml_diff>